<commit_message>
change xls source to xlsx DB sec
</commit_message>
<xml_diff>
--- a/NAV 구성종목시세_20260421_182930.xlsx
+++ b/NAV 구성종목시세_20260421_182930.xlsx
@@ -5,22 +5,22 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\uv\kis_ws\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\git\etftracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CEB2FB6-1B75-4A1A-9B2F-5F60F6662E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF6BADB-CADE-4D64-A71A-624B667BD2DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9450" yWindow="8535" windowWidth="17700" windowHeight="10605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8610" yWindow="3345" windowWidth="19620" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="118">
   <si>
     <t>종목명</t>
   </si>
@@ -374,15 +374,15 @@
   </si>
   <si>
     <t>−</t>
-  </si>
-  <si>
-    <t>J010010</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -451,7 +451,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -460,6 +460,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="백분율" xfId="1" builtinId="5"/>
@@ -817,8 +818,8 @@
       <c r="F2">
         <v>700</v>
       </c>
-      <c r="G2" s="3">
-        <v>7.4507138409970086E-2</v>
+      <c r="G2" s="4">
+        <v>7.4507138409970084</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -846,8 +847,8 @@
       <c r="F3">
         <v>780</v>
       </c>
-      <c r="G3" s="3">
-        <v>6.9951264449854764E-2</v>
+      <c r="G3" s="4">
+        <v>6.995126444985476</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
@@ -875,8 +876,8 @@
       <c r="F4">
         <v>120</v>
       </c>
-      <c r="G4" s="3">
-        <v>4.1124404720006218E-2</v>
+      <c r="G4" s="4">
+        <v>4.112440472000622</v>
       </c>
       <c r="H4" t="s">
         <v>16</v>
@@ -904,8 +905,8 @@
       <c r="F5">
         <v>91</v>
       </c>
-      <c r="G5" s="3">
-        <v>3.6950642258162497E-2</v>
+      <c r="G5" s="4">
+        <v>3.6950642258162496</v>
       </c>
       <c r="H5" t="s">
         <v>18</v>
@@ -933,8 +934,8 @@
       <c r="F6">
         <v>120</v>
       </c>
-      <c r="G6" s="3">
-        <v>3.6174449503842132E-2</v>
+      <c r="G6" s="4">
+        <v>3.617444950384213</v>
       </c>
       <c r="H6" t="s">
         <v>20</v>
@@ -962,8 +963,8 @@
       <c r="F7">
         <v>500</v>
       </c>
-      <c r="G7" s="3">
-        <v>3.4620222494004878E-2</v>
+      <c r="G7" s="4">
+        <v>3.462022249400488</v>
       </c>
       <c r="H7" t="s">
         <v>22</v>
@@ -991,8 +992,8 @@
       <c r="F8">
         <v>119</v>
       </c>
-      <c r="G8" s="3">
-        <v>3.3418642963295407E-2</v>
+      <c r="G8" s="4">
+        <v>3.3418642963295406</v>
       </c>
       <c r="H8" t="s">
         <v>24</v>
@@ -1020,8 +1021,8 @@
       <c r="F9">
         <v>49</v>
       </c>
-      <c r="G9" s="3">
-        <v>3.3296183133728847E-2</v>
+      <c r="G9" s="4">
+        <v>3.3296183133728849</v>
       </c>
       <c r="H9" t="s">
         <v>26</v>
@@ -1049,8 +1050,8 @@
       <c r="F10">
         <v>149</v>
       </c>
-      <c r="G10" s="3">
-        <v>3.2624219347129779E-2</v>
+      <c r="G10" s="4">
+        <v>3.2624219347129779</v>
       </c>
       <c r="H10" t="s">
         <v>29</v>
@@ -1078,8 +1079,8 @@
       <c r="F11">
         <v>179</v>
       </c>
-      <c r="G11" s="3">
-        <v>2.9205104075607499E-2</v>
+      <c r="G11" s="4">
+        <v>2.9205104075607498</v>
       </c>
       <c r="H11" t="s">
         <v>31</v>
@@ -1107,8 +1108,8 @@
       <c r="F12">
         <v>350</v>
       </c>
-      <c r="G12" s="3">
-        <v>2.8520249780633011E-2</v>
+      <c r="G12" s="4">
+        <v>2.8520249780633011</v>
       </c>
       <c r="H12" t="s">
         <v>33</v>
@@ -1136,8 +1137,8 @@
       <c r="F13">
         <v>100</v>
       </c>
-      <c r="G13" s="3">
-        <v>2.4712946056890721E-2</v>
+      <c r="G13" s="4">
+        <v>2.4712946056890721</v>
       </c>
       <c r="H13" t="s">
         <v>35</v>
@@ -1165,8 +1166,8 @@
       <c r="F14">
         <v>89</v>
       </c>
-      <c r="G14" s="3">
-        <v>2.4485704809243902E-2</v>
+      <c r="G14" s="4">
+        <v>2.4485704809243902</v>
       </c>
       <c r="H14" t="s">
         <v>37</v>
@@ -1194,8 +1195,8 @@
       <c r="F15">
         <v>300</v>
       </c>
-      <c r="G15" s="3">
-        <v>2.3865855506505489E-2</v>
+      <c r="G15" s="4">
+        <v>2.3865855506505489</v>
       </c>
       <c r="H15" t="s">
         <v>39</v>
@@ -1223,8 +1224,8 @@
       <c r="F16">
         <v>199</v>
       </c>
-      <c r="G16" s="3">
-        <v>2.2280691276567229E-2</v>
+      <c r="G16" s="4">
+        <v>2.228069127656723</v>
       </c>
       <c r="H16" t="s">
         <v>41</v>
@@ -1252,8 +1253,8 @@
       <c r="F17">
         <v>249</v>
       </c>
-      <c r="G17" s="3">
-        <v>2.1711575331792111E-2</v>
+      <c r="G17" s="4">
+        <v>2.171157533179211</v>
       </c>
       <c r="H17" t="s">
         <v>43</v>
@@ -1281,8 +1282,8 @@
       <c r="F18">
         <v>149</v>
       </c>
-      <c r="G18" s="3">
-        <v>2.12921734342916E-2</v>
+      <c r="G18" s="4">
+        <v>2.1292173434291599</v>
       </c>
       <c r="H18" t="s">
         <v>45</v>
@@ -1310,8 +1311,8 @@
       <c r="F19">
         <v>69</v>
       </c>
-      <c r="G19" s="3">
-        <v>2.0914665689011229E-2</v>
+      <c r="G19" s="4">
+        <v>2.0914665689011227</v>
       </c>
       <c r="H19" t="s">
         <v>47</v>
@@ -1339,8 +1340,8 @@
       <c r="F20">
         <v>180</v>
       </c>
-      <c r="G20" s="3">
-        <v>1.9225272491351648E-2</v>
+      <c r="G20" s="4">
+        <v>1.9225272491351648</v>
       </c>
       <c r="H20" t="s">
         <v>49</v>
@@ -1368,8 +1369,8 @@
       <c r="F21">
         <v>80</v>
       </c>
-      <c r="G21" s="3">
-        <v>1.745743134272161E-2</v>
+      <c r="G21" s="4">
+        <v>1.745743134272161</v>
       </c>
       <c r="H21" t="s">
         <v>51</v>
@@ -1397,8 +1398,8 @@
       <c r="F22">
         <v>49</v>
       </c>
-      <c r="G22" s="3">
-        <v>1.7514333729693139E-2</v>
+      <c r="G22" s="4">
+        <v>1.7514333729693139</v>
       </c>
       <c r="H22" t="s">
         <v>53</v>
@@ -1426,8 +1427,8 @@
       <c r="F23">
         <v>100</v>
       </c>
-      <c r="G23" s="3">
-        <v>1.738377129486203E-2</v>
+      <c r="G23" s="4">
+        <v>1.7383771294862029</v>
       </c>
       <c r="H23" t="s">
         <v>55</v>
@@ -1455,8 +1456,8 @@
       <c r="F24">
         <v>59</v>
       </c>
-      <c r="G24" s="3">
-        <v>1.6938312155431189E-2</v>
+      <c r="G24" s="4">
+        <v>1.693831215543119</v>
       </c>
       <c r="H24" t="s">
         <v>57</v>
@@ -1484,8 +1485,8 @@
       <c r="F25">
         <v>100</v>
       </c>
-      <c r="G25" s="3">
-        <v>1.6702415852160861E-2</v>
+      <c r="G25" s="4">
+        <v>1.6702415852160861</v>
       </c>
       <c r="H25" t="s">
         <v>59</v>
@@ -1513,8 +1514,8 @@
       <c r="F26">
         <v>80</v>
       </c>
-      <c r="G26" s="3">
-        <v>1.633779861525592E-2</v>
+      <c r="G26" s="4">
+        <v>1.6337798615255921</v>
       </c>
       <c r="H26" t="s">
         <v>61</v>
@@ -1542,8 +1543,8 @@
       <c r="F27">
         <v>29</v>
       </c>
-      <c r="G27" s="3">
-        <v>1.5326814458383121E-2</v>
+      <c r="G27" s="4">
+        <v>1.532681445838312</v>
       </c>
       <c r="H27" t="s">
         <v>63</v>
@@ -1571,8 +1572,8 @@
       <c r="F28">
         <v>100</v>
       </c>
-      <c r="G28" s="3">
-        <v>1.4695179547987181E-2</v>
+      <c r="G28" s="4">
+        <v>1.4695179547987181</v>
       </c>
       <c r="H28" t="s">
         <v>65</v>
@@ -1600,8 +1601,8 @@
       <c r="F29">
         <v>120</v>
       </c>
-      <c r="G29" s="3">
-        <v>1.3789160959314281E-2</v>
+      <c r="G29" s="4">
+        <v>1.3789160959314282</v>
       </c>
       <c r="H29" t="s">
         <v>67</v>
@@ -1629,8 +1630,8 @@
       <c r="F30">
         <v>150</v>
       </c>
-      <c r="G30" s="3">
-        <v>1.36455238659881E-2</v>
+      <c r="G30" s="4">
+        <v>1.3645523865988101</v>
       </c>
       <c r="H30" t="s">
         <v>69</v>
@@ -1658,8 +1659,8 @@
       <c r="F31">
         <v>150</v>
       </c>
-      <c r="G31" s="3">
-        <v>1.276160329167308E-2</v>
+      <c r="G31" s="4">
+        <v>1.276160329167308</v>
       </c>
       <c r="H31" t="s">
         <v>71</v>
@@ -1687,8 +1688,8 @@
       <c r="F32">
         <v>149</v>
       </c>
-      <c r="G32" s="3">
-        <v>1.278627940770604E-2</v>
+      <c r="G32" s="4">
+        <v>1.278627940770604</v>
       </c>
       <c r="H32" t="s">
         <v>73</v>
@@ -1716,8 +1717,8 @@
       <c r="F33">
         <v>300</v>
       </c>
-      <c r="G33" s="3">
-        <v>1.2457755594252291E-2</v>
+      <c r="G33" s="4">
+        <v>1.2457755594252291</v>
       </c>
       <c r="H33" t="s">
         <v>75</v>
@@ -1745,8 +1746,8 @@
       <c r="F34">
         <v>49</v>
       </c>
-      <c r="G34" s="3">
-        <v>1.1179937914008139E-2</v>
+      <c r="G34" s="4">
+        <v>1.117993791400814</v>
       </c>
       <c r="H34" t="s">
         <v>77</v>
@@ -1774,8 +1775,8 @@
       <c r="F35">
         <v>199</v>
       </c>
-      <c r="G35" s="3">
-        <v>1.1030408016853181E-2</v>
+      <c r="G35" s="4">
+        <v>1.1030408016853182</v>
       </c>
       <c r="H35" t="s">
         <v>79</v>
@@ -1803,8 +1804,8 @@
       <c r="F36">
         <v>50</v>
       </c>
-      <c r="G36" s="3">
-        <v>9.9441064610439559E-3</v>
+      <c r="G36" s="4">
+        <v>0.99441064610439556</v>
       </c>
       <c r="H36" t="s">
         <v>81</v>
@@ -1832,8 +1833,8 @@
       <c r="F37">
         <v>9</v>
       </c>
-      <c r="G37" s="3">
-        <v>9.9606799718123615E-3</v>
+      <c r="G37" s="4">
+        <v>0.99606799718123618</v>
       </c>
       <c r="H37" t="s">
         <v>83</v>
@@ -1861,8 +1862,8 @@
       <c r="F38">
         <v>30</v>
       </c>
-      <c r="G38" s="3">
-        <v>9.8833369215597985E-3</v>
+      <c r="G38" s="4">
+        <v>0.98833369215597988</v>
       </c>
       <c r="H38" t="s">
         <v>85</v>
@@ -1890,8 +1891,8 @@
       <c r="F39">
         <v>50</v>
       </c>
-      <c r="G39" s="3">
-        <v>9.8796539191668194E-3</v>
+      <c r="G39" s="4">
+        <v>0.98796539191668198</v>
       </c>
       <c r="H39" t="s">
         <v>87</v>
@@ -1919,8 +1920,8 @@
       <c r="F40">
         <v>11</v>
       </c>
-      <c r="G40" s="3">
-        <v>9.7838958569493577E-3</v>
+      <c r="G40" s="4">
+        <v>0.97838958569493573</v>
       </c>
       <c r="H40" t="s">
         <v>89</v>
@@ -1948,8 +1949,8 @@
       <c r="F41">
         <v>233</v>
       </c>
-      <c r="G41" s="3">
-        <v>9.6755235115359439E-3</v>
+      <c r="G41" s="4">
+        <v>0.96755235115359439</v>
       </c>
       <c r="H41" t="s">
         <v>91</v>
@@ -1977,8 +1978,8 @@
       <c r="F42">
         <v>200</v>
       </c>
-      <c r="G42" s="3">
-        <v>9.5021461738864464E-3</v>
+      <c r="G42" s="4">
+        <v>0.95021461738864466</v>
       </c>
       <c r="H42" t="s">
         <v>93</v>
@@ -2006,8 +2007,8 @@
       <c r="F43">
         <v>100</v>
       </c>
-      <c r="G43" s="3">
-        <v>8.968110826904456E-3</v>
+      <c r="G43" s="4">
+        <v>0.89681108269044563</v>
       </c>
       <c r="H43" t="s">
         <v>95</v>
@@ -2035,8 +2036,8 @@
       <c r="F44">
         <v>15</v>
       </c>
-      <c r="G44" s="3">
-        <v>8.5077355277820513E-3</v>
+      <c r="G44" s="4">
+        <v>0.8507735527782051</v>
       </c>
       <c r="H44" t="s">
         <v>97</v>
@@ -2064,8 +2065,8 @@
       <c r="F45">
         <v>200</v>
       </c>
-      <c r="G45" s="3">
-        <v>8.2683403722384006E-3</v>
+      <c r="G45" s="4">
+        <v>0.82683403722384008</v>
       </c>
       <c r="H45" t="s">
         <v>99</v>
@@ -2093,8 +2094,8 @@
       <c r="F46">
         <v>45</v>
       </c>
-      <c r="G46" s="3">
-        <v>7.6735354857722527E-3</v>
+      <c r="G46" s="4">
+        <v>0.76735354857722526</v>
       </c>
       <c r="H46" t="s">
         <v>101</v>
@@ -2122,8 +2123,8 @@
       <c r="F47">
         <v>29</v>
       </c>
-      <c r="G47" s="3">
-        <v>7.1667543564983083E-3</v>
+      <c r="G47" s="4">
+        <v>0.71667543564983083</v>
       </c>
       <c r="H47" t="s">
         <v>103</v>
@@ -2151,8 +2152,8 @@
       <c r="F48">
         <v>100</v>
       </c>
-      <c r="G48" s="3">
-        <v>6.6846493432573253E-3</v>
+      <c r="G48" s="4">
+        <v>0.66846493432573251</v>
       </c>
       <c r="H48" t="s">
         <v>105</v>
@@ -2180,8 +2181,8 @@
       <c r="F49">
         <v>15</v>
       </c>
-      <c r="G49" s="3">
-        <v>6.5741592714679484E-3</v>
+      <c r="G49" s="4">
+        <v>0.65741592714679487</v>
       </c>
       <c r="H49" t="s">
         <v>107</v>
@@ -2209,8 +2210,8 @@
       <c r="F50">
         <v>150</v>
       </c>
-      <c r="G50" s="3">
-        <v>6.2288777971261436E-3</v>
+      <c r="G50" s="4">
+        <v>0.62288777971261433</v>
       </c>
       <c r="H50" t="s">
         <v>109</v>
@@ -2238,8 +2239,8 @@
       <c r="F51">
         <v>161</v>
       </c>
-      <c r="G51" s="3">
-        <v>4.654762574366816E-3</v>
+      <c r="G51" s="4">
+        <v>0.46547625743668158</v>
       </c>
       <c r="H51" t="s">
         <v>111</v>
@@ -2267,8 +2268,8 @@
       <c r="F52">
         <v>100</v>
       </c>
-      <c r="G52" s="3">
-        <v>3.434399731453144E-3</v>
+      <c r="G52" s="4">
+        <v>0.34343997314531438</v>
       </c>
       <c r="H52" t="s">
         <v>113</v>
@@ -2296,8 +2297,8 @@
       <c r="F53">
         <v>147</v>
       </c>
-      <c r="G53" s="3">
-        <v>2.4606691437853269E-3</v>
+      <c r="G53" s="4">
+        <v>0.2460669143785327</v>
       </c>
       <c r="H53" t="s">
         <v>115</v>
@@ -2325,11 +2326,8 @@
       <c r="F54">
         <v>6440686</v>
       </c>
-      <c r="G54" s="3">
-        <v>1.1860530975213951E-2</v>
-      </c>
-      <c r="H54" t="s">
-        <v>118</v>
+      <c r="G54" s="4">
+        <v>1.186053097521395</v>
       </c>
       <c r="I54">
         <v>6440686</v>

</xml_diff>